<commit_message>
deploy: 118 pins / 16 countries (AITHYRA, AI BioDesign, CircuLab, BESSY III) + regenerated analytics
</commit_message>
<xml_diff>
--- a/sdl-data.xlsx
+++ b/sdl-data.xlsx
@@ -9499,6 +9499,339 @@
         </is>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">aithyra</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AITHYRA</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Austrian Academy of Sciences (ÖAW) · Vienna BioCenter</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vienna</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Austria</t>
+        </is>
+      </c>
+      <c r="F116">
+        <v>48.19</v>
+      </c>
+      <c r="G116">
+        <v>16.4</v>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">academic</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">biology</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prototype</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">single-technique</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">strong</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AI-driven robotics lab · 100 m² phase I → 400 m² phase II · 10–14 groups</t>
+        </is>
+      </c>
+      <c r="N116">
+        <v>150</v>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">€150M / 12 yrs (Boehringer Ingelheim Stiftung)</t>
+        </is>
+      </c>
+      <c r="P116">
+        <v>2024</v>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://aithyra.at/</t>
+        </is>
+      </c>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://aithyra.at/research/research-at-aithyra ; https://aithyra.at/research/groups/wali-malik ; https://boehringer-ingelheim-stiftung.de/en/what-we-fund/funding-initiatives/aithyra-institute.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">allen_biodesign</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AI BioDesign (Allen Institute)</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Allen Institute + UW + Fred Hutch · Fund for Science and Technology</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seattle</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USA</t>
+        </is>
+      </c>
+      <c r="F117">
+        <v>47.62</v>
+      </c>
+      <c r="G117">
+        <v>-122.34</v>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">academic</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">biology</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">operational</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">single-technique</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">strong</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accelerator · massively parallel in-tube libraries (scale not from robotics)</t>
+        </is>
+      </c>
+      <c r="N117">
+        <v>95</v>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$95M (FFST)</t>
+        </is>
+      </c>
+      <c r="P117">
+        <v>2026</v>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://alleninstitute.org/</t>
+        </is>
+      </c>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://alleninstitute.org/news/ai-biodesign-accelerator-combines-experimental-biology-and-artificial-intelligence-to-learn-natures-design-rules ; https://www.eurekalert.org/news-releases/1141802</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">circulab</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CircuLab</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stockholm University · WISE Research Technology Platform</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stockholm</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sweden</t>
+        </is>
+      </c>
+      <c r="F118">
+        <v>59.37</v>
+      </c>
+      <c r="G118">
+        <v>18.05</v>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">academic</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">materials</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">operational</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">multi-technique</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">strong</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 clusters · ~20 instruments · open to academia, start-ups, industry</t>
+        </is>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WISE + Stockholm University (part of SEK 136M over 4 platforms)</t>
+        </is>
+      </c>
+      <c r="P118">
+        <v>2024</v>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://wise-materials.org/platform/circulab</t>
+        </is>
+      </c>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://wise-materials.org/platform/circulab ; https://www.su.se/english/news/articles/2026-08-17-launch-of-the-wise-research-technology-platfrom-circulab ; https://www.su.se/english/news/articles/2024-01-17-sek-136-millions-granted-to-materials-research-at-stockholm-university</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bessy3</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BESSY III</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Helmholtz-Zentrum Berlin (HZB)</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Berlin</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Germany</t>
+        </is>
+      </c>
+      <c r="F119">
+        <v>52.43</v>
+      </c>
+      <c r="G119">
+        <v>13.53</v>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">national</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">materials</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">concept</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">advanced-multimodal</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">planned</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4th-gen soft X-ray source · CDR 2027 · operations mid-2030s</t>
+        </is>
+      </c>
+      <c r="N119">
+        <v>900</v>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">≈€900M construction (est., 2020 prices)</t>
+        </is>
+      </c>
+      <c r="P119">
+        <v>2022</v>
+      </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.helmholtz-berlin.de/forschung/quellen/bessy3/index_en.html</t>
+        </is>
+      </c>
+      <c r="R119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.helmholtz-berlin.de/media/landing/bessy3/index.html ; https://jacow.org/icalepcs2023/papers/mo2ao04.pdf ; https://pmc.ncbi.nlm.nih.gov/articles/PMC10119534</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -9519,14 +9852,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">114 initiatives across 15 countries</t>
+          <t xml:space="preserve">118 initiatives across 16 countries</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dataset as of 2026-09-09</t>
+          <t xml:space="preserve">Dataset as of 2026-09-15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploy: brand motto, about page, SEO pass
</commit_message>
<xml_diff>
--- a/sdl-data.xlsx
+++ b/sdl-data.xlsx
@@ -66,6 +66,7 @@
     <col min="16" max="16" width="12" customWidth="1"/>
     <col min="17" max="17" width="40" customWidth="1"/>
     <col min="18" max="18" width="60" customWidth="1"/>
+    <col min="19" max="19" width="80" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -159,6 +160,11 @@
           <t xml:space="preserve">sources</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blurb</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -243,6 +249,11 @@
           <t xml:space="preserve">https://acceleration.utoronto.ca/vision ; https://acceleration.utoronto.ca/facilities</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">200-member global consortium anchoring 30+ self-driving labs for sustainable materials and molecules across health, energy, and electronics.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -327,6 +338,11 @@
           <t xml:space="preserve">https://dg.dk/en/centers/pioneer-center-for-accelerating-p2x-materials-discovery-capex/ ; https://www.dtu.dk/english/newsarchive/2022/12/power-to-x-center-vil-revolutionere-materialer-til-den-groenne-omstilling</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Danish 13-year Pioneer Center accelerating Power-to-X catalyst and material discovery across DTU, Aalborg, Stanford, SLAC, Utrecht, and Toronto.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -411,6 +427,11 @@
           <t xml:space="preserve">https://battery2030.eu/battery2030/projects/big-map/ ; https://www.full-map.eu/ ; https://battery2030.eu/</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Battery2030+ flagship Materials Acceleration Platform for battery interfaces. BIG-MAP closed Feb 2024; successor FULL-MAP runs 2025-2029.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -495,6 +516,11 @@
           <t xml:space="preserve">https://arpa-e.energy.gov/news-and-events/news-and-insights/us-department-energy-announces-34-million-pair-artificial-intelligence-autonomous-labs-accelerate-catalyst-development-0 ; https://science.osti.gov/</t>
         </is>
       </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">US federal SDL funding through ARPA-E's $40M catalyst programme and CHIPS R&amp;D's $100M semiconductor-materials programme for autonomous chemistry and electronics discovery.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -579,6 +605,11 @@
           <t xml:space="preserve">https://pubs.rsc.org/en/content/articlelanding/2025/dd/d6dd00024j</t>
         </is>
       </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOTIE's October 2024 AI+R&amp;D Strategy commits Korea to 500 autonomous laboratories by 2030 across nanomaterials, catalysis, organic chemistry, and bioengineering.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -663,6 +694,11 @@
           <t xml:space="preserve">https://news.nus.edu.sg/ai-for-science-nus-4-ai-based-projects/</t>
         </is>
       </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Singapore's National Research Foundation AI4S programme (launched June 2026); NUS leads four of eight inaugural projects, anchored by the Materials Data Foundry (Novoselov + Aspuru-Guzik, I-FIM) building an open AI-and-robotics autonomous lab to link synthesis protocols to real-world material performance.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -747,6 +783,11 @@
           <t xml:space="preserve">https://aria.org.uk/funding-opportunities/ ; https://aria.org.uk/about-aria/</t>
         </is>
       </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARIA programme funding 12 AI Scientist projects testing autonomous hypothesis-to-experiment systems across drugs, batteries, quantum dots, and biology.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -826,6 +867,11 @@
           <t xml:space="preserve">https://discoverylabs.nl/</t>
         </is>
       </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dutch shared infrastructure linking DIFFER and three TU/e institutes for autonomous materials discovery, targeting NWO LSRI submission in 2027.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -910,6 +956,11 @@
           <t xml:space="preserve">https://www.bigchemistry-nijmegen.nl/ ; https://www.ru.nl/en/research/research-projects/robot-lab-for-big-chemistry-in-the-netherlands</t>
         </is>
       </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dutch National Growth Fund consortium of five institutes (Radboud lead, TU/e, Groningen, AMOLF, Fontys) building AI-guided self-driving labs for sustainable industrial formulations.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -994,6 +1045,11 @@
           <t xml:space="preserve">https://www.cnrs.fr/en/pepr/emerging-materials-diadem ; https://www.sciencedirect.com/science/article/pii/S2001037024003052</t>
         </is>
       </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">France 2030 programme run by CNRS, CEA, and seven academic partners, funding 51 projects that fuse AI with synthesis and characterisation across France.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1075,6 +1131,11 @@
           <t xml:space="preserve">https://doi.org/10.1038/s41586-023-06734-w ; https://newscenter.lbl.gov/2023/04/17/meet-the-autonomous-lab-of-the-future/</t>
         </is>
       </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Closed-loop robotic synthesis, characterisation, and ML-driven decision-making for inorganic solid-state materials, targeting 10-100x faster discovery.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1156,6 +1217,11 @@
           <t xml:space="preserve">https://www.anl.gov/article/argonnes-selfdriving-lab-accelerates-the-discovery-process-for-materials-with-multiple-applications ; https://spectrum.ieee.org/autonomous-lab-argonne-polybot</t>
         </is>
       </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AI-driven autonomous platform at Argonne CNM that synthesises, prints, and tests electronic polymer films for solar cells, biosensors, and recyclable devices.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1237,6 +1303,11 @@
           <t xml:space="preserve">https://www.cmu.edu/mcs/research/cloud-lab/index.html ; https://www.cmu.edu/news/stories/archives/2021/august/first-academic-cloud-lab.html</t>
         </is>
       </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Remote-access 24/7 facility with 200+ instruments letting researchers anywhere design and run autonomous chemistry, biology, and materials experiments.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1318,6 +1389,11 @@
           <t xml:space="preserve">https://doi.org/10.1038/s41586-023-06792-0 ; https://www.cmu.edu/news/stories/archives/2023/december/cmu-designed-artificially-intelligent-coscientist-automates-scientific-discovery</t>
         </is>
       </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LLM-driven agent from Gabe Gomes' group that reads literature, plans syntheses, and controls liquid-handling robots from natural-language prompts.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1399,6 +1475,11 @@
           <t xml:space="preserve">https://cbe.ncsu.edu/abolhasani-hit-fast-forward/ ; https://research.ncsu.edu/nc-state-receives-3m-from-arpa-e-to-advance-self-driving-laboratory-research/</t>
         </is>
       </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Self-driving fluidic lab combining microreactor flow chemistry, robotics, and AI to accelerate perovskite quantum dots and energy-relevant materials.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1483,6 +1564,11 @@
           <t xml:space="preserve">https://www.chalmers.se/en/departments/cse/our-research/data-science-and-ai/king-lab/ ; https://research.chalmers.se/en/person/rossk</t>
         </is>
       </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ross King's third-generation Robot Scientist programme pursuing fully automated hypothesis generation and testing across biology and chemistry.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1567,6 +1653,11 @@
           <t xml:space="preserve">https://www.liverpool.ac.uk/cooper-group/</t>
         </is>
       </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Andy Cooper's mobile robot chemists roam the Materials Innovation Factory, autonomously running photocatalyst, porous-material, and CO₂-capture experiments; the £81M MIF opened in 2017, building on the robotic Centre for Materials Discovery running since 2007.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1648,6 +1739,11 @@
           <t xml:space="preserve">https://www.helmholtz.de/en/research/research-fields/matter/ ; https://www.helmholtz.de/en/newsroom/article/a-revolution-with-ai-and-robotics/</t>
         </is>
       </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KIT-led Helmholtz consortium positioning Germany's autonomous SDLs for health, energy storage, catalysis, and electronics in smart data centres.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1732,6 +1828,11 @@
           <t xml:space="preserve">https://cnsi.ucla.edu/nsf-biopacific-mip/ ; https://www.sharedinstrumentation.ucsb.edu/facilities/california-nanosystems-institute/biopacific-mip</t>
         </is>
       </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NSF Materials Innovation Platform at UCSB and UCLA offering free peer-reviewed access to automated, AI-driven synthesis and characterisation of bio-derived materials.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1816,6 +1917,11 @@
           <t xml:space="preserve">https://www.eu-startups.com/2025/09/british-startup-cuspai-secures-e85-million-to-transform-materials-discovery-with-ai</t>
         </is>
       </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AI-driven materials discovery startup (Max Welling co-founder) designing functional crystals on demand for carbon capture, batteries, PFAS removal, and semiconductors.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1897,6 +2003,11 @@
           <t xml:space="preserve">https://www.eu-startups.com/2025/09/british-startup-cuspai-secures-e85-million-to-transform-materials-discovery-with-ai</t>
         </is>
       </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Amsterdam Science Park (Lab42) node of CuspAI running the Welling-led ML stack for generative inverse design of functional materials.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1978,6 +2089,11 @@
           <t xml:space="preserve">https://doi.org/10.1021/acs.accounts.4c00095 ; https://www.solar.fau.de/2024/04/23/toward-self-driven-autonomous-material-and-device-acceleration-platforms-amadap-for-emerging-photovoltaics-technologies/</t>
         </is>
       </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brabec group platform spanning high-throughput synthesis, SPINBOT spin-coating, and the AMANDA device line to autonomously discover emerging photovoltaic materials.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2059,6 +2175,11 @@
           <t xml:space="preserve">https://www.nims.go.jp/eng/press/2025/12/202512100.html ; https://doi.org/10.1038/s41524-025-01851-8</t>
         </is>
       </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NIMS-Tsukuba framework letting multiple autonomous AI labs spontaneously share data and coordinate searches across different material systems.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2140,6 +2261,11 @@
           <t xml:space="preserve">https://pubs.rsc.org/en/content/articlehtml/2025/dd/d4dd00387j</t>
         </is>
       </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hitosugi-group digital lab chaining thin-film synthesis with XRD, Raman, conductivity, and optics for fully automated standardised materials data.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2221,6 +2347,11 @@
           <t xml:space="preserve">https://www.theengineer.co.uk/content/news/ai-lab-speeds-battery-cathode-discovery ; https://www.miragenews.com/ai-robotic-arms-achieve-material-breakthrough-1512230/</t>
         </is>
       </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dong-Hwa Seo's industry-academia autonomous lab with POSCO N.EX.T Hub cutting battery cathode discovery time by 93 percent.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2302,6 +2433,11 @@
           <t xml:space="preserve">https://www.kist.re.kr/eng/research/materials-latest-research-news.do?mode=view&amp;articleNo=13112 ; https://www.eurekalert.org/news-releases/1042809</t>
         </is>
       </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KIST's robotic synthesis + characterisation + ML workflow for accelerated discovery across battery and functional materials.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2383,6 +2519,11 @@
           <t xml:space="preserve">https://www.chem.ubc.ca/ubc-s-hein-lab-and-seoul-national-university-partnership-expanding-self-driving-labs-clean-energy</t>
         </is>
       </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yousung Jung's group uses LLMs to predict material synthesisability, anchoring a wider SNU autonomous-lab cluster across batteries and catalysis.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2464,6 +2605,11 @@
           <t xml:space="preserve">http://staff.ustc.edu.cn/~jiangj1/ ; https://doi.org/10.1038/s44286-024-00139-w ; https://www.nature.com/articles/s44286-022-00018-3</t>
         </is>
       </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Robotic AI-Chemist 2.0 lineage couples on-board LLM multi-agent ChemAgents with cloud-linked lab robots for autonomous chemistry.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2545,6 +2691,11 @@
           <t xml:space="preserve">https://www.uva.nl/en/profile/n/o/t.noel/t.noel.html</t>
         </is>
       </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flow chemistry group running RoboChem, an autonomous photocatalytic reaction platform that optimises continuous-flow photochemistry without human intervention.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2626,6 +2777,11 @@
           <t xml:space="preserve">https://www.differ.nl/research/autonomous-energy-materials-discovery ; https://www.amdlab.nl/</t>
         </is>
       </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Computational group screening energy materials (redox-flow electrolytes, electrocatalysts) via high-throughput DFT plus ML over public chemical databases.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2710,6 +2866,11 @@
           <t xml:space="preserve">https://www.flagshippioneering.com/news/press-release/flagship-pioneering-unveils-lila-sciences-to-build-superintelligence-in-science ; https://www.lila.ai/about</t>
         </is>
       </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flagship Pioneering venture building Scientific Superintelligence: AI agents coupled to autonomous wet labs across therapeutics, materials, energy, and chemicals.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2794,6 +2955,11 @@
           <t xml:space="preserve">https://www.medra.ai/about ; https://www.businesswire.com/news/home/20251211748411/en/Medra-Raises-$52-Million-Series-A-to-Build-Physical-AI-Scientists ; https://www.medra.ai/medra-lab-001</t>
         </is>
       </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Physical AI scientists for life-science labs: vision-guided robot arms operating standard instruments end-to-end across gene editing, cell biology, and microbial discovery.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2875,6 +3041,11 @@
           <t xml:space="preserve">https://techcrunch.com/2025/10/20/top-openai-google-brain-researchers-set-off-a-300m-vc-frenzy-for-their-startup-periodic-labs/</t>
         </is>
       </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stealth-emerged lab building AI scientists with paired autonomous laboratories, starting with materials physics: superconductors and semiconductor thermal materials.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2959,6 +3130,11 @@
           <t xml:space="preserve">https://en.xtalpi.com/about/ ; https://en.wikipedia.org/wiki/XtalPi</t>
         </is>
       </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HKEX-listed AI + quantum-physics + robotics platform running autonomous drug-discovery and materials labs across Shenzhen, Shanghai, and Boston.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3040,6 +3216,11 @@
           <t xml:space="preserve">https://labgeniustx.com/sanofi/</t>
         </is>
       </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bermondsey biotech whose EVA platform closed-loops ML design with automated wet-lab cycles to engineer selectivity-enhanced antibodies for solid tumours.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3121,6 +3302,11 @@
           <t xml:space="preserve">http://hjkgrp.mit.edu/post/26-03-31-heather-deep-principle/ ; https://www.weforum.org/organizations/deep-principle/</t>
         </is>
       </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Agentic AI for materials and chemistry. ECML framework orchestrates DFT, MD, ML, and wet-lab experiments; recently hired MIT's Heather Kulik as Chief Scientist.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3197,6 +3383,11 @@
           <t xml:space="preserve">https://www.quiktech.cn/</t>
         </is>
       </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Beijing-registered robotics-plus-AI scale-up building chemistry workstations for pharma, energy, and advanced materials; planning a 100-robot AI cloud lab in Yichang.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3278,6 +3469,11 @@
           <t xml:space="preserve">https://www.ylab.ac.cn/en/about_us/ ; https://www.ylab.ac.cn/en/news/yJ_news/03-18/1555490091.html</t>
         </is>
       </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Zhejiang provincial materials research institute running advanced functional, structural, and transformative materials platforms including a 6-inch micro-nano device line.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3359,6 +3555,11 @@
           <t xml:space="preserve">https://bohrium.dp.tech/en-US ; https://www.dp.tech/en/about</t>
         </is>
       </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AI-for-Science company behind Bohrium, Hermite, Piloteye, and Uni-Lab, building foundation-model infrastructure for chemistry, biology, and batteries.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3435,6 +3636,11 @@
           <t xml:space="preserve">https://www.ikkem.com/</t>
         </is>
       </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Provincial mega-institute building China's first dedicated energy-storage research infrastructure, spanning low-carbon energy, displays, and graphene.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3516,6 +3722,11 @@
           <t xml:space="preserve">https://open-sciencelab.github.io/index.html</t>
         </is>
       </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">National AGI lab whose AGI4S programme builds Intern-S1 scientific foundation models and the Intern-Discovery agent-plus-instrument platform.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3597,6 +3808,11 @@
           <t xml:space="preserve">https://seed.bytedance.com/en/ ; https://seed.bytedance.com/en/research</t>
         </is>
       </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ByteDance's foundation-model team applying AI to biological structure prediction (Protenix), quantum chemistry, and topological materials physics.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3678,6 +3894,11 @@
           <t xml:space="preserve">https://arxiv.org/abs/2406.10536 ; https://hyper.ai/en/news/32891</t>
         </is>
       </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tsinghua physics group developing DeepH, a universal neural-network DFT Hamiltonian model accelerating electronic-structure prediction across arbitrary material structures.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3759,6 +3980,11 @@
           <t xml:space="preserve">https://chemrxiv.org/engage/api-gateway/chemrxiv/assets/orp/resource/item/6447d756e4bbbe4bbf3afeaa/original/metal-organic-frameworks-meet-uni-mof-a-revolutionary-gas-adsorption-detector.pdf</t>
         </is>
       </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Xiaonan Wang's group building foundation models (SurFF, Uni-MOF) for catalyst surfaces and MOF gas adsorption at high-throughput screening scale.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3840,6 +4066,11 @@
           <t xml:space="preserve">https://doi.org/10.1021/acs.jmedchem.3c02029 ; https://www.chemspeed.com/news/microcycle/</t>
         </is>
       </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Novartis Basel in-house self-driving lab integrating micro-scale synthesis, automated purification, real-time bioassays, and ML-driven compound design.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3921,6 +4152,11 @@
           <t xml:space="preserve">https://ir.bruker.com/press-releases/press-release-details/2024/Bruker-Announces-Closing-of-Chemspeed-Technologies-AG-Acquisition/default.aspx ; https://www.sciy.com/</t>
         </is>
       </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Swiss lab-automation vendor selling modular robotic synthesis, formulation, and characterisation workflows for materials, pharma, and battery R&amp;D.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4002,6 +4238,11 @@
           <t xml:space="preserve">https://www.isc.fraunhofer.de/en.html ; https://doi.org/10.1002/adma.202407791</t>
         </is>
       </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fraunhofer ISC programme coupling robotic synthesis and characterisation with AI-driven design for glass, battery, and functional materials.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4083,6 +4324,11 @@
           <t xml:space="preserve">https://en.wikipedia.org/wiki/Emerald_Cloud_Lab</t>
         </is>
       </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Remote-controlled cloud laboratory letting scientists design and run wet-lab experiments on 200+ instrument models via a unified software interface.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4167,6 +4413,11 @@
           <t xml:space="preserve">https://www.ginkgo.bio/autonomous-lab ; https://www.ginkgo.bio/about</t>
         </is>
       </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Synthetic-biology platform offering autonomous strain-engineering foundries and cloud-lab access for antibody, enzyme, and cell-line programmes.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4248,6 +4499,11 @@
           <t xml:space="preserve">https://ai-science-foundry.cmu.edu/about-ai-science-foundry ; https://www.cmu.edu/future-of-science/cloud-lab/index.html</t>
         </is>
       </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carnegie Mellon initiative running the ASAP autonomous platform for AI-guided experiments in hard materials, chemistry, and biology.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4329,6 +4585,11 @@
           <t xml:space="preserve">https://strateos.com/virtual-lab-tour/ ; https://investor.lilly.com/news-releases/news-release-details/eli-lilly-and-company-collaboration-strateos-inc-launch-remote</t>
         </is>
       </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cloud-lab-as-a-service operating robotic San Diego and Menlo Park facilities for remote small-molecule, biologics, and synthetic-biology workflows.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4413,6 +4674,11 @@
           <t xml:space="preserve">https://www.kebotix.com/about-us</t>
         </is>
       </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Self-driving lab platform pairing generative chemistry, automated synthesis, and robotic characterisation for specialty-chemicals and advanced-materials discovery.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4497,6 +4763,11 @@
           <t xml:space="preserve">https://www.arctoris.com/about-us/ ; https://www.arctoris.com/arctoris-automated-platform-accelerates-drug-discovery/</t>
         </is>
       </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oxford-based automated drug-discovery CRO running the Ulysses robotic platform for reproducible biochemical, cell, and molecular assay data.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4581,6 +4852,11 @@
           <t xml:space="preserve">https://www.prnewswire.com/news-releases/culture-biosciences-unveils-stratyx-250-the-first-cloud-integrated-mobile-bioreactor-for-cell-culture-process-development-302415306.html</t>
         </is>
       </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cloud-connected 250 mL bioreactor service for outsourced upstream bioprocess development with remote monitoring and bioprocess software.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4665,6 +4941,11 @@
           <t xml:space="preserve">https://www.automata.tech/linq ; https://www.moleculardevices.com/newsroom/news/molecular-devices-partnership-with-automata-linq-platform</t>
         </is>
       </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LINQ platform orchestrates modular benchtop robotics with a node-based workflow canvas and Python SDK for genomics and assay screening.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4749,6 +5030,11 @@
           <t xml:space="preserve">https://www.benchling.com/about-us</t>
         </is>
       </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cloud R&amp;D platform combining ELN, registry, inventory, and workflow tools for biotech, used by most large biopharma.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4830,6 +5116,11 @@
           <t xml:space="preserve">https://www.fiercebiotech.com/medtech/microsoft-leads-21m-investment-artificial-s-automation-platform-for-life-science-labs</t>
         </is>
       </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">aLab Suite orchestrates instruments, robots, people, and data into closed-loop digital workflows for life-science labs (Palo Alto, USA · Microsoft M12-backed).</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4911,6 +5202,11 @@
           <t xml:space="preserve">https://www.synthace.com/about ; https://www.synthace.com/how-it-works</t>
         </is>
       </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Digital experiment platform for designing, simulating, and executing high-dimensional multivariate experiments on lab automation hardware.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4992,6 +5288,11 @@
           <t xml:space="preserve">https://www.unchainedlabs.com/stuntman/ ; https://www.prnewswire.com/news-releases/unchained-labs-explodes-into-ai-driven-automation-launches-stuntman-302681892.html</t>
         </is>
       </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stuntman is a natural-language AI automation platform with flexible hardware for biologics, gene therapy, and reaction screening.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5073,6 +5374,11 @@
           <t xml:space="preserve">https://www.munich-startup.de/en/startups/unitelabs/ ; https://sila-standard.com/sila_device/unitelabs-connectivity-platform/</t>
         </is>
       </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Python-based lab automation OS connecting 175+ instruments through one API for code-defined, version-controlled workflows.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5154,6 +5460,11 @@
           <t xml:space="preserve">https://www.cenevo.com/about ; https://www.cenevo.com/press/labguru-and-titian-software-rebrand-as-cenevo</t>
         </is>
       </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Post-merger entity behind Mosaic sample tracking and Labguru ELN/LIMS, integrating 150+ instruments across biopharma R&amp;D.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5235,6 +5546,11 @@
           <t xml:space="preserve">https://opentrons.com/</t>
         </is>
       </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Modular robotic workcells and Cellario scheduling software paired with Opentrons via a 2026 agent-to-agent AI workflow partnership.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5316,6 +5632,11 @@
           <t xml:space="preserve">https://atinary.com/technology/sdlabs/ ; https://www.chemspeed.com/news/atinaryxchemspeed/</t>
         </is>
       </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SDLabs no-code platform pairing Bayesian and ML optimizers with robotic hardware for closed-loop chemistry and materials discovery.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5397,6 +5718,11 @@
           <t xml:space="preserve">https://global.abb/group/en/ ; https://new.abb.com/locations/group-headquarters</t>
         </is>
       </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Industrial robotics arm supplying GoFa and YuMi collaborative arms plus AVR autonomous mobile robots for multi-vendor lab workcells.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5478,6 +5804,11 @@
           <t xml:space="preserve">https://cheme.mit.edu/profile/klavs-f-jensen/ ; https://news.mit.edu/2018/technology-automates-chemical-synthesis-0920</t>
         </is>
       </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIT ChemE group integrating flow reactors, robotics, online analytics, and machine learning into autonomous platforms for reaction discovery and process development.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5559,6 +5890,11 @@
           <t xml:space="preserve">https://www.chemify.io/ ; https://www.chemify.io/about</t>
         </is>
       </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Glasgow group behind the Chemputer and chemputation: synthesis encoded as executable code on universal robotic platforms, commercialised through spinout Chemify.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5640,6 +5976,11 @@
           <t xml:space="preserve">https://scholar.google.com/citations?user=hjS0xZ0AAAAJ&amp;hl=pl</t>
         </is>
       </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IBS Center for Algorithmic and Robotized Synthesis pairing AI retrosynthesis (Chematica/Synthia) with closed-loop chemical robotics.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5724,6 +6065,11 @@
           <t xml:space="preserve">https://burke-group.chemistry.illinois.edu/about/ ; https://chemistry.illinois.edu/news/2025-07-30/nsf-reinvests-molecule-maker-lab-institute-ai-tools-solve-chemistrys-challenges</t>
         </is>
       </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NSF-funded institute around Burke's iterative MIDA-boronate small-molecule synthesizer, closing the loop with AI agents like AlphaSynthesis.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5805,6 +6151,11 @@
           <t xml:space="preserve">https://telescopeinnovations.com/ ; http://hein.chem.ubc.ca/</t>
         </is>
       </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UBC spinout commercialising self-driving process-chemistry platforms (IvoryOS, DirectInject-LC) for pharma, critical minerals, and Acceleration Consortium partners.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5886,6 +6237,11 @@
           <t xml:space="preserve">https://www.ch.cam.ac.uk/person/svl1000</t>
         </is>
       </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cambridge group pioneering continuous-flow and machine-assisted synthesis for natural products and methodology, with four spinouts and 900+ publications.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5967,6 +6323,11 @@
           <t xml:space="preserve">https://www.doylelab.com/ ; https://www.chemistry.ucla.edu/directory/doyle-abigail</t>
         </is>
       </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UCLA catalysis group fusing nickel cross-coupling, photocatalysis, and machine-learning reaction optimisation through founding roles in BioLEC and C-CAS centres.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6048,6 +6409,11 @@
           <t xml:space="preserve">https://www.hamiltoncompany.com/about-us</t>
         </is>
       </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reno-based manufacturer of Microlab liquid-handling robots, process sensors, and automated sample-storage systems used across pharma and clinical labs.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6132,6 +6498,11 @@
           <t xml:space="preserve">https://en.wikipedia.org/wiki/Opentrons</t>
         </is>
       </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open-source liquid-handling robots and the Flex workstation plus OpentronsAI natural-language protocol design for genomics and proteomics labs.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6213,6 +6584,11 @@
           <t xml:space="preserve">https://lifesciences.tecan.com/products/liquid_handling_and_automation</t>
         </is>
       </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Swiss-listed maker of Fluent and Freedom EVO liquid-handling platforms plus OEM components for diagnostics and life-science automation.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -6294,6 +6670,11 @@
           <t xml:space="preserve">https://grenova.com/paa-automation/ ; https://grenova.com/paa-joins-grenovas-parent-company-to-advance-lab-automation/</t>
         </is>
       </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UK lab-automation integrator building modular robotic workcells with Overlord scheduling software for life-science and pharma throughput.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6378,6 +6759,11 @@
           <t xml:space="preserve">https://www.princeton.edu/news/2025/08/20/princeton-tapped-partner-new-nsf-funded-ai-materials-institute</t>
         </is>
       </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First NSF AI institute dedicated to materials, coordinating closed-loop autonomous experimentation across Cornell, Princeton, CCNY, and Boston University.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6462,6 +6848,11 @@
           <t xml:space="preserve">https://www.governor.ny.gov/news/governor-hochul-celebrates-radical-ai-establishing-new-yorks-first-fully-autonomous-materials</t>
         </is>
       </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AI agents coupled to a closed-loop robotic lab discovering inorganic materials, alloys, and electrolytes; CSO Gerbrand Ceder built LBNL's A-Lab.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6546,6 +6937,11 @@
           <t xml:space="preserve">https://cen.acs.org/articles/103/web/2025/11/Mattiq-quest-make-billions-nanomaterials.html</t>
         </is>
       </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Northwestern spinout running high-throughput combinatorial megalibrary synthesis of millions of nanomaterials per day to train AI for clean-energy catalysts.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6627,6 +7023,11 @@
           <t xml:space="preserve">https://nrc.canada.ca/en/research-development/research-collaboration/programs/critical-battery-materials-initiative</t>
         </is>
       </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">National Research Council Canada self-driving labs for battery-materials discovery and critical-mineral processing under the Critical Battery Materials Initiative.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6711,6 +7112,11 @@
           <t xml:space="preserve">https://news.liverpool.ac.uk/2024/02/06/liverpool-and-imperial-college-london-to-lead-uks-flagship-12m-ai-for-chemistry-hub/</t>
         </is>
       </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">£12M EPSRC national hub (Liverpool + Imperial) developing AI-planned robotic and autonomous chemistry, including mobile robot scientists for exploratory synthesis.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6795,6 +7201,11 @@
           <t xml:space="preserve">https://tech.eu/2026/05/20/dunia-innovations-unveils-eur280m-berlin-gigalab-to-industrialise-ai-driven-materials-discovery/</t>
         </is>
       </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Self-driving labs running the full design-make-test-analyse loop for electrocatalyst, battery, and CO2-conversion materials, scaling to a €280M Berlin GigaLab.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6876,6 +7287,11 @@
           <t xml:space="preserve">https://www.ncbi.nlm.nih.gov/pmc/articles/PMC12067375/</t>
         </is>
       </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Modular robotic platform integrating automated synthesis, characterisation, and evaluation, demonstrated on metal-halide perovskites.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6957,6 +7373,11 @@
           <t xml:space="preserve">https://www.kit.edu/kit/english/pi_2022_011_battery-research-first-fully-automatic-laboratory-starts-operation.php</t>
         </is>
       </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fully automated, AI-planned battery-materials lab that autonomously synthesises, assembles, and cycles cells.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7038,6 +7459,11 @@
           <t xml:space="preserve">https://pubs.acs.org/doi/10.1021/acsnano.4c17504</t>
         </is>
       </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Self-driving platform for nano- and advanced-materials synthesis with active-learning optimisation.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7122,6 +7548,11 @@
           <t xml:space="preserve">https://technode.global/2025/12/08/ai-for-science-startup-chemlex-raises-45m-launching-self-driving-lab-for-drug-discovery-in-singapore/</t>
         </is>
       </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24/7 fully automated robotic synthesis line (~800 reactions/day) coupling AI to wet-lab chemistry for drug discovery.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7206,6 +7637,11 @@
           <t xml:space="preserve">https://pubs.rsc.org/en/content/articlehtml/2025/dd/d4dd00387j</t>
         </is>
       </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JST-funded national self-driving lab (Maholo robotic-arm platform) for closed-loop materials discovery, with a prototyping lab at RIKEN BDR Kobe and a demonstrator at Institute of Science Tokyo.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7287,6 +7723,11 @@
           <t xml:space="preserve">https://pubs.rsc.org/en/content/articlehtml/2025/dd/d4dd00387j</t>
         </is>
       </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AIST's Multi-Modal AI lab-automation initiative for autonomous experimentation, now spanning all seven AIST research departments.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7368,6 +7809,11 @@
           <t xml:space="preserve">https://pubs.rsc.org/en/content/articlehtml/2026/dd/d6dd00024j</t>
         </is>
       </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Closed-loop alloy discovery (arc-melting to annealing to XRD) with reinforcement-learning optimisation.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -7449,6 +7895,11 @@
           <t xml:space="preserve">https://pubs.rsc.org/en/content/articlehtml/2026/dd/d6dd00024j</t>
         </is>
       </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24-hour autonomous synthesis, analysis, and XRD for safety-critical energy and catalyst materials.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7533,6 +7984,11 @@
           <t xml:space="preserve">https://www.crunchbase.com/organization/megarobo</t>
         </is>
       </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">China's largest smart-lab robotics company, building autonomous agents that run real experiments across life sciences, chemistry, and energy materials.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7617,6 +8073,11 @@
           <t xml:space="preserve">https://techcrunch.com/2025/05/01/futurehouse-releases-ai-tools-it-claims-can-accelerate-science/</t>
         </is>
       </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AI-scientist agent stack (the Robin multi-agent discovery system) coupled to its own robotic wet lab; for-profit spinout Edison.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7701,6 +8162,11 @@
           <t xml:space="preserve">https://ascend-project.berlin/news/a-new-era-in-catalysis-ascend-launch-in-berlin-e30-million-in-funding/ ; https://www.helmholtz-berlin.de/</t>
         </is>
       </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BMFTR-funded consortium led by Helmholtz-Zentrum Berlin and the Fritz Haber Institute (with BASF, Siemens Energy, Dunia Innovations, and TU Berlin/BasCat) running AI-guided self-driving labs, high-throughput characterisation, and digital twins to accelerate catalyst discovery for sustainable chemistry.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7782,6 +8248,11 @@
           <t xml:space="preserve">https://www.tsinghua.edu.cn/en/info/1244/14984.htm ; https://www.nature.com/articles/d41586-026-02143-x ; https://www.nytimes.com/2026/07/09/science/nobel-winning-us-chemist-will-move-to-china-to-lead-ai-institute.html</t>
         </is>
       </c>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Institute announced in 2026 at Tsinghua University, to be led by Nobel laureate Omar Yaghi, pairing AI with reticular chemistry for materials discovery; at concept stage, with no facility details public yet.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7866,6 +8337,11 @@
           <t xml:space="preserve">https://www.nsf.gov/tip/updates/nsf-announces-400m-investment-new-national-network-ai ; https://www.nsf.gov/funding/opportunities/pcl-test-bed-test-bed-toward-network-programmable-cloud-laboratories ; https://www.psu.edu/news/research/story/penn-state-awarded-20m-lead-nsf-programmable-cloud-laboratory</t>
         </is>
       </c>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NSF national network of AI-enabled programmable cloud laboratories: ~$380M to 20 teams over four years plus Astera Institute matching, anchored by nodes like Penn State's LATTICE thin-film SDL with Argonne.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -7950,6 +8426,11 @@
           <t xml:space="preserve">https://www.solvechemistry.com/ ; https://www.linkedin.com/company/solve-chemistry/</t>
         </is>
       </c>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">London SDL flow lab pairing online-UHPLC high-throughput experimentation with Bayesian optimisation for predictive process chemistry and right-first-time scale-up.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -8031,6 +8512,11 @@
           <t xml:space="preserve">https://mission-innovation.net/press-release-materials-workshop-report/ ; https://www.science.org/doi/10.1126/scirobotics.aat5559 ; https://pubs.acs.org/acscii/article/4/2/144/733253/The-Matter-Simulation-R-evolution</t>
         </is>
       </c>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alán Aspuru-Guzik's group; originated the modern SDL field with ChemOS (2017) and spun out Kebotix, Atinary, and the Acceleration Consortium.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -8112,6 +8598,11 @@
           <t xml:space="preserve">https://www.youtube.com/watch?v=tWub0OgBGhE</t>
         </is>
       </c>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Haranczyk group self-driving lab for automated polymer processing (melt and solution workflows), serving six Madrid research groups and the Materials-Commons EU network.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -8196,6 +8687,11 @@
           <t xml:space="preserve">https://imms.ewha.ac.kr/en/news/83 ; https://www.hankyung.com/article/2026072665561</t>
         </is>
       </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Korea's MSIT / NRL 2.0 national research laboratory at Ewha Womans University (director Hoi Ri Moon); a 330 m² self-driving lab with ten function-based workstations across five material classes, a Bayesian-optimisation and LLM-agent decision layer, moving to open-access user operation from 2028.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -8277,6 +8773,11 @@
           <t xml:space="preserve">https://doi.org/10.1002/ange.202214511 ; https://doi.org/10.1016/j.cej.2022.138443</t>
         </is>
       </c>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Institute of Process Research and Development, University of Leeds.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -8358,6 +8859,11 @@
           <t xml:space="preserve">https://www.epfl.ch/research/facilities/swisscat/publications-patents-conference-participation/ ; https://ch.linkedin.com/company/swisscatpluseast ; https://www.chimia.ch/chimia/article/view/2023_154</t>
         </is>
       </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ETH Domain-funded national catalysis infrastructure jointly operated by EPFL and ETH Zurich, combining robotic high-throughput experimentation, AI-guided experimental design, and automated workflows to enable self-driving laboratories for catalyst discovery and optimization across homogeneous and heterogeneous catalysis.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -8439,6 +8945,11 @@
           <t xml:space="preserve">https://doi.org/10.1016/j.xcrp.2025.102548 ; https://urn.kb.se/resolve?urn=urn:nbn:se:uu:diva-578031 ; https://doi.org/10.5281/zenodo.14191482</t>
         </is>
       </c>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Self-driving battery laboratory developed at Uppsala University's Ångström Advanced Battery Centre, integrating automated electrolyte formulation, robotic coin-cell assembly, in-line cycling, computer vision, and Bayesian optimization for closed-loop electrolyte discovery.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -8520,6 +9031,11 @@
           <t xml:space="preserve">https://doi.org/10.1002/batt.202500155 ; https://pubs.rsc.org/doi/d5dd00567a ; https://zenodo.org/records/15481956</t>
         </is>
       </c>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Battaglia Lab's autonomous robotic battery-materials platform automating electrolyte formulation, cell assembly, and cycling on &gt;1200 cycler channels, with ontologized FAIR data management.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -8601,6 +9117,11 @@
           <t xml:space="preserve">https://doi.org/10.1038/s41929-024-01172-x ; https://www.empa.ch/web/s604/parallel-co2-electrolysis</t>
         </is>
       </c>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Battaglia Lab platform running 8 parallel CO₂-electrolysis reactors for gas-diffusion electrodes with automated online gas and liquid product analysis, published as an open blueprint.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -8682,6 +9203,11 @@
           <t xml:space="preserve">https://doi.org/10.1038/npjcompumats.2016.31 ; https://doi.org/10.1038/s41570-026-00847-2</t>
         </is>
       </c>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Air Force Research Laboratory's Autonomous Research System (Maruyama): ARES OS was the first major infrastructure package for SDL deployment, demonstrated on autonomous carbon-nanotube growth.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -8763,6 +9289,11 @@
           <t xml:space="preserve">https://doi.org/10.1038/s41467-020-19597-w ; https://doi.org/10.1038/s41570-026-00847-2</t>
         </is>
       </c>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NIST's closed-loop autonomous system (Kusne) running Bayesian phase mapping jointly with property optimisation live on synchrotron beamlines, with opt-in human collaboration.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -8844,6 +9375,11 @@
           <t xml:space="preserve">https://doi.org/10.1021/acsnano.4c17504 ; https://doi.org/10.1038/s41570-026-00847-2</t>
         </is>
       </c>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BAM's modular robotic platform (Rühle group) for synthesis, purification, and in-line characterisation of nano- and advanced materials (seven materials across five classes), with ELN/LIMS integration via OpenBIS.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -8925,6 +9461,11 @@
           <t xml:space="preserve">https://doi.org/10.1126/sciadv.aaz1708 ; https://doi.org/10.1038/s41570-026-00847-2</t>
         </is>
       </c>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Keith Brown's Bayesian experimental autonomous researcher: closed-loop additive manufacturing and mechanical-design experiments, one of the field's flagship SDL architectures.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -9006,6 +9547,11 @@
           <t xml:space="preserve">https://doi.org/10.1038/s41467-020-15728-5 ; https://doi.org/10.1038/s41570-026-00847-2</t>
         </is>
       </c>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The first cloud-SDL demonstration: Xi Zhu's materials acceleration operating system in cloud, which autonomously discovered chiral inorganic perovskite nanocrystals via remote collaboration.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -9090,6 +9636,11 @@
           <t xml:space="preserve">https://ai4science.sg/ ; https://www.a-star.edu.sg/imre/research-departments/electronic-materials-department/accelerated-catalyst-development-platform-(acdp)</t>
         </is>
       </c>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kedar Hippalgaonkar's initiative integrating AI, robotics, and agentically driven high-throughput experiments for functional energy and electronic materials, backed by a S$25M MTI Programmatic Award and the S$10M Mat-GDT platform.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -9174,6 +9725,11 @@
           <t xml:space="preserve">https://raeng.org.uk/programmes-and-prizes/programmes/uk-grants-and-prizes/support-for-research/research-awardees/research-fellowships-awardees/2024-2029/dr-connor-taylor/ ; https://pmc.ncbi.nlm.nih.gov/articles/PMC10214532/</t>
         </is>
       </c>
+      <c r="S111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Connor Taylor's self-driving laboratory for drug discovery and chemical process development, funded through a £2M RAEng research fellowship.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -9255,6 +9811,11 @@
           <t xml:space="preserve">https://cicenergigune.com/es/noticias/cicenergigune-descubrimiento-nuevos-inteligencia-artificial ; https://doi.org/10.1039/d4dd00381k ; https://doi.org/10.1107/S1600576724006885</t>
         </is>
       </c>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Automation and AI platform for inorganic energy materials combining automated co-precipitation, solvothermal, and sol-gel synthesis with XRD and electrochemical characterisation and active-learning experiment design.</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -9336,6 +9897,11 @@
           <t xml:space="preserve">https://sila-standard.com/interview-with-iacob-marian-from-qpillars/</t>
         </is>
       </c>
+      <c r="S113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Zurich startup making lab instruments agent-ready through MCP servers and SiLA 2 drivers, so AI copilots can turn natural-language requests into validated, reproducible instrument workflows.</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -9417,6 +9983,11 @@
           <t xml:space="preserve">https://www.siat.ac.cn/cxpt/202412/t20241214_7458457.html ; https://www.siat.ac.cn/symt/202604/t20260416_8186608.html</t>
         </is>
       </c>
+      <c r="S114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAS SIAT-led national major science infrastructure at Guangming Science City: modular fully-automated workcells running the synthetic-biology design-build-test-learn loop at high throughput, open to academic and industrial users.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -9498,6 +10069,11 @@
           <t xml:space="preserve">https://hic.zju.edu.cn/ibct/58279/list.htm ; http://hic.zju.edu.cn/82840/list.htm</t>
         </is>
       </c>
+      <c r="S115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Zhejiang University's twin automated science installations at the Hangzhou Innovation Center — a synthetic-biology iBioFoundry and a molecular-manufacturing iChemFoundry, 300+ instruments across 14,000 m², operated as shared platforms.</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -9582,6 +10158,11 @@
           <t xml:space="preserve">https://aithyra.at/research/research-at-aithyra ; https://aithyra.at/research/groups/wali-malik ; https://boehringer-ingelheim-stiftung.de/en/what-we-fund/funding-initiatives/aithyra-institute.html</t>
         </is>
       </c>
+      <c r="S116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Austrian Academy of Sciences institute for biomedical AI under founding director Michael Bronstein, building a closed-loop AI-driven robotics lab: vision-enabled liquid handlers, self-teaching robotic arms, and sensor-rich work cells under an AI orchestration layer, with 100 m² in phase I at the Marxbox and 400 m² in the purpose-built Vienna BioCenter building.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -9666,6 +10247,11 @@
           <t xml:space="preserve">https://alleninstitute.org/news/ai-biodesign-accelerator-combines-experimental-biology-and-artificial-intelligence-to-learn-natures-design-rules ; https://www.eurekalert.org/news-releases/1141802</t>
         </is>
       </c>
+      <c r="S117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open-science accelerator with the University of Washington and Fred Hutch designing proteins and genes that do not exist in nature; bench teams run massively parallel library experiments while a machine-learning team chooses each next round, scored on how much the models improved. Scale comes from parallelising inside the test tube rather than from robotics.</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -9747,6 +10333,11 @@
           <t xml:space="preserve">https://wise-materials.org/platform/circulab ; https://www.su.se/english/news/articles/2026-08-17-launch-of-the-wise-research-technology-platfrom-circulab ; https://www.su.se/english/news/articles/2024-01-17-sek-136-millions-granted-to-materials-research-at-stockholm-university</t>
         </is>
       </c>
+      <c r="S118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WISE Research Technology Platform at Stockholm University for circular and sustainable materials: automated synthesis and processing, real-time monitoring of emissions, hazardous chemicals and physicochemical change, and ML plus Bayesian-optimisation decision making across four clusters and about 20 instruments; open to academia, start-ups, and industry.</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -9829,6 +10420,11 @@
       <c r="R119" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.helmholtz-berlin.de/media/landing/bessy3/index.html ; https://jacow.org/icalepcs2023/papers/mo2ao04.pdf ; https://pmc.ncbi.nlm.nih.gov/articles/PMC10119534</t>
+        </is>
+      </c>
+      <c r="S119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HZB's 4th-generation soft-to-tender X-ray source for Berlin-Adlershof, planned from the ground up around intelligent autonomous experimentation, AI-supported sample synthesis and handling, and FAIR data, with synthesis and characterisation laboratories on the same integrated research campus; CDR due 2027, construction from 2032, operations mid-2030s.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploy 6e124ae: Claim & Connect
</commit_message>
<xml_diff>
--- a/sdl-data.xlsx
+++ b/sdl-data.xlsx
@@ -67,6 +67,10 @@
     <col min="17" max="17" width="40" customWidth="1"/>
     <col min="18" max="18" width="60" customWidth="1"/>
     <col min="19" max="19" width="80" customWidth="1"/>
+    <col min="20" max="20" width="12" customWidth="1"/>
+    <col min="21" max="21" width="12" customWidth="1"/>
+    <col min="22" max="22" width="12" customWidth="1"/>
+    <col min="23" max="23" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -165,6 +169,26 @@
           <t xml:space="preserve">blurb</t>
         </is>
       </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">open_offers</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">open_seeks</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stack</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">maintained_with_lab</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1658,6 +1682,11 @@
           <t xml:space="preserve">Andy Cooper's mobile robot chemists roam the Materials Innovation Factory, autonomously running photocatalyst, porous-material, and CO₂-capture experiments; the £81M MIF opened in 2017, building on the robotic Centre for Materials Discovery running since 2007.</t>
         </is>
       </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4157,6 +4186,11 @@
           <t xml:space="preserve">Swiss lab-automation vendor selling modular robotic synthesis, formulation, and characterisation workflows for materials, pharma, and battery R&amp;D.</t>
         </is>
       </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6675,6 +6709,11 @@
           <t xml:space="preserve">UK lab-automation integrator building modular robotic workcells with Overlord scheduling software for life-science and pharma throughput.</t>
         </is>
       </c>
+      <c r="W76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -8431,6 +8470,11 @@
           <t xml:space="preserve">London SDL flow lab pairing online-UHPLC high-throughput experimentation with Bayesian optimisation for predictive process chemistry and right-first-time scale-up.</t>
         </is>
       </c>
+      <c r="W96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -8517,6 +8561,11 @@
           <t xml:space="preserve">Alán Aspuru-Guzik's group; originated the modern SDL field with ChemOS (2017) and spun out Kebotix, Atinary, and the Acceleration Consortium.</t>
         </is>
       </c>
+      <c r="W97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -8603,6 +8652,11 @@
           <t xml:space="preserve">Haranczyk group self-driving lab for automated polymer processing (melt and solution workflows), serving six Madrid research groups and the Materials-Commons EU network.</t>
         </is>
       </c>
+      <c r="W98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -8692,6 +8746,11 @@
           <t xml:space="preserve">Korea's MSIT / NRL 2.0 national research laboratory at Ewha Womans University (director Hoi Ri Moon); a 330 m² self-driving lab with ten function-based workstations across five material classes, a Bayesian-optimisation and LLM-agent decision layer, moving to open-access user operation from 2028.</t>
         </is>
       </c>
+      <c r="W99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -8778,6 +8837,11 @@
           <t xml:space="preserve">Institute of Process Research and Development, University of Leeds.</t>
         </is>
       </c>
+      <c r="W100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-07</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -8864,6 +8928,11 @@
           <t xml:space="preserve">ETH Domain-funded national catalysis infrastructure jointly operated by EPFL and ETH Zurich, combining robotic high-throughput experimentation, AI-guided experimental design, and automated workflows to enable self-driving laboratories for catalyst discovery and optimization across homogeneous and heterogeneous catalysis.</t>
         </is>
       </c>
+      <c r="W101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-07</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -8950,6 +9019,11 @@
           <t xml:space="preserve">Self-driving battery laboratory developed at Uppsala University's Ångström Advanced Battery Centre, integrating automated electrolyte formulation, robotic coin-cell assembly, in-line cycling, computer vision, and Bayesian optimization for closed-loop electrolyte discovery.</t>
         </is>
       </c>
+      <c r="W102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -9036,6 +9110,11 @@
           <t xml:space="preserve">Battaglia Lab's autonomous robotic battery-materials platform automating electrolyte formulation, cell assembly, and cycling on &gt;1200 cycler channels, with ontologized FAIR data management.</t>
         </is>
       </c>
+      <c r="W103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -9122,6 +9201,11 @@
           <t xml:space="preserve">Battaglia Lab platform running 8 parallel CO₂-electrolysis reactors for gas-diffusion electrodes with automated online gas and liquid product analysis, published as an open blueprint.</t>
         </is>
       </c>
+      <c r="W104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -9641,6 +9725,11 @@
           <t xml:space="preserve">Kedar Hippalgaonkar's initiative integrating AI, robotics, and agentically driven high-throughput experiments for functional energy and electronic materials, backed by a S$25M MTI Programmatic Award and the S$10M Mat-GDT platform.</t>
         </is>
       </c>
+      <c r="W110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -9730,6 +9819,11 @@
           <t xml:space="preserve">Connor Taylor's self-driving laboratory for drug discovery and chemical process development, funded through a £2M RAEng research fellowship.</t>
         </is>
       </c>
+      <c r="W111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -9816,6 +9910,11 @@
           <t xml:space="preserve">Automation and AI platform for inorganic energy materials combining automated co-precipitation, solvothermal, and sol-gel synthesis with XRD and electrochemical characterisation and active-learning experiment design.</t>
         </is>
       </c>
+      <c r="W112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -9900,6 +9999,11 @@
       <c r="S113" t="inlineStr">
         <is>
           <t xml:space="preserve">Zurich startup making lab instruments agent-ready through MCP servers and SiLA 2 drivers, so AI copilots can turn natural-language requests into validated, reproducible instrument workflows.</t>
+        </is>
+      </c>
+      <c r="W113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08</t>
         </is>
       </c>
     </row>
@@ -10455,7 +10559,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dataset as of 2026-09-27</t>
+          <t xml:space="preserve">Dataset as of 2026-10-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploy 6d309ec: DiscoveryLabNL entry reframed (TU/e-coordinated)
</commit_message>
<xml_diff>
--- a/sdl-data.xlsx
+++ b/sdl-data.xlsx
@@ -826,7 +826,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">NWO LSRI</t>
+          <t xml:space="preserve">TU/e</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dutch shared infrastructure linking DIFFER and three TU/e institutes for autonomous materials discovery, targeting NWO LSRI submission in 2027.</t>
+          <t xml:space="preserve">Dutch national infrastructure for AI-driven materials discovery, coordinated by TU/e and starting with energy materials.</t>
         </is>
       </c>
     </row>
@@ -10559,7 +10559,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dataset as of 2026-10-11</t>
+          <t xml:space="preserve">Dataset as of 2026-10-12</t>
         </is>
       </c>
     </row>

</xml_diff>